<commit_message>
v2 fix some bugs
</commit_message>
<xml_diff>
--- a/weekly_report.xlsx
+++ b/weekly_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\develop\05_report_tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26A2DEA-FBE7-4BE5-9F27-B7651ACB4420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{538116DB-1423-4234-8520-07A17707FB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7752" yWindow="1656" windowWidth="14028" windowHeight="11208" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="report" sheetId="1" r:id="rId1"/>
@@ -351,6 +351,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -358,24 +376,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -668,13 +668,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="9"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="15"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -682,19 +682,19 @@
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="9" t="s">
         <v>5</v>
       </c>
       <c r="F2" s="2"/>
@@ -704,7 +704,7 @@
       <c r="J2" s="2"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="10" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -721,7 +721,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="14"/>
+      <c r="A4" s="11"/>
       <c r="B4" s="3" t="s">
         <v>10</v>
       </c>
@@ -736,21 +736,21 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="14"/>
+      <c r="A5" s="11"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="4"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="14"/>
+      <c r="A6" s="11"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="4"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="11" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -767,7 +767,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="14"/>
+      <c r="A8" s="11"/>
       <c r="B8" s="3" t="s">
         <v>12</v>
       </c>
@@ -782,21 +782,21 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
+      <c r="A9" s="11"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="4"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="14"/>
+      <c r="A10" s="11"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="4"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="11" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -813,7 +813,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
+      <c r="A12" s="11"/>
       <c r="B12" s="3" t="s">
         <v>14</v>
       </c>
@@ -828,14 +828,14 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="14"/>
+      <c r="A13" s="11"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="4"/>
     </row>
     <row r="14" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="15"/>
+      <c r="A14" s="12"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
@@ -850,5 +850,6 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>